<commit_message>
Fix fallvignette export processing refs #1328
</commit_message>
<xml_diff>
--- a/R-dataprocessor/submodules/manual_start/Fallvignette_Process_Evaluation/R-Fallvignette_Process_Evaluation/inst/extdata/WP8MRP_Liste_Daten_Mapping20260722.xlsx
+++ b/R-dataprocessor/submodules/manual_start/Fallvignette_Process_Evaluation/R-Fallvignette_Process_Evaluation/inst/extdata/WP8MRP_Liste_Daten_Mapping20260722.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{EE6A06D7-04C5-4693-89AC-F1482AA91ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7BDE5A9-AD65-4507-AC16-D90695611332}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{EE6A06D7-04C5-4693-89AC-F1482AA91ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E97DF81-D74D-4470-8A66-A9D79154D81D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="111">
   <si>
     <t>Fallvignette</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>Standortübergreifend eindeutig</t>
+  </si>
+  <si>
+    <t>wp8_ret_id</t>
+  </si>
+  <si>
+    <t>ret_id</t>
   </si>
   <si>
     <t>wp8_standort_id</t>
@@ -752,7 +758,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D98"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="13.15"/>
   <cols>
     <col min="1" max="1" width="54.85546875" customWidth="1"/>
@@ -787,15 +793,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" ht="12.75">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -805,6 +808,9 @@
       <c r="B4" t="s">
         <v>10</v>
       </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
@@ -813,15 +819,15 @@
       <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
         <v>14</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>15</v>
       </c>
     </row>
@@ -841,31 +847,30 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="12.75" customHeight="1">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="B9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" ht="12.75" customHeight="1">
       <c r="A10" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="3"/>
+      <c r="D10" s="3" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D11" s="3"/>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" t="s">
         <v>25</v>
       </c>
       <c r="D12" s="3"/>
@@ -874,9 +879,10 @@
       <c r="A13" t="s">
         <v>26</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>27</v>
       </c>
+      <c r="D13" s="3"/>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
@@ -1094,31 +1100,31 @@
         <v>81</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="24">
+    <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>36</v>
+        <v>82</v>
       </c>
       <c r="B41" t="s">
-        <v>82</v>
-      </c>
-      <c r="D41" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="12.75">
+    <row r="42" spans="1:4" ht="24">
       <c r="A42" t="s">
         <v>38</v>
       </c>
       <c r="B42" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="43" spans="1:4">
+      <c r="D42" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="12.75">
       <c r="A43" t="s">
         <v>40</v>
       </c>
       <c r="B43" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -1126,7 +1132,7 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -1134,7 +1140,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -1142,7 +1148,7 @@
         <v>46</v>
       </c>
       <c r="B46" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -1150,7 +1156,7 @@
         <v>48</v>
       </c>
       <c r="B47" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -1158,7 +1164,7 @@
         <v>50</v>
       </c>
       <c r="B48" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -1166,7 +1172,7 @@
         <v>52</v>
       </c>
       <c r="B49" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -1174,7 +1180,7 @@
         <v>54</v>
       </c>
       <c r="B50" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -1182,7 +1188,7 @@
         <v>56</v>
       </c>
       <c r="B51" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -1190,7 +1196,7 @@
         <v>58</v>
       </c>
       <c r="B52" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -1198,7 +1204,7 @@
         <v>60</v>
       </c>
       <c r="B53" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -1206,7 +1212,7 @@
         <v>62</v>
       </c>
       <c r="B54" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -1214,7 +1220,7 @@
         <v>64</v>
       </c>
       <c r="B55" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -1222,7 +1228,7 @@
         <v>66</v>
       </c>
       <c r="B56" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -1230,7 +1236,7 @@
         <v>68</v>
       </c>
       <c r="B57" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -1238,7 +1244,7 @@
         <v>70</v>
       </c>
       <c r="B58" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -1246,7 +1252,7 @@
         <v>72</v>
       </c>
       <c r="B59" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -1254,7 +1260,7 @@
         <v>74</v>
       </c>
       <c r="B60" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -1262,7 +1268,7 @@
         <v>76</v>
       </c>
       <c r="B61" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -1270,7 +1276,7 @@
         <v>78</v>
       </c>
       <c r="B62" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -1278,30 +1284,38 @@
         <v>80</v>
       </c>
       <c r="B63" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="70" spans="2:4">
-      <c r="B70" t="s">
+        <v>82</v>
+      </c>
+      <c r="B64" t="s">
         <v>107</v>
       </c>
-      <c r="D70" t="s">
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="97" spans="3:3">
-      <c r="C97" t="s">
-        <v>106</v>
+    <row r="71" spans="1:4">
+      <c r="B71" t="s">
+        <v>109</v>
+      </c>
+      <c r="D71" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="98" spans="3:3">
+      <c r="C98" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="D9:D12"/>
+    <mergeCell ref="D10:D13"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -1313,6 +1327,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -1362,32 +1385,7 @@
 </spe:Receivers>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="93d2b372-37bc-474e-a2f6-e237b07f4f3a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_dlc_DocId xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f">TMFEV-885672295-4175</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f">
-      <Url>https://tmfev.sharepoint.com/sites/tmf/mi-i/_layouts/15/DocIdRedir.aspx?ID=TMFEV-885672295-4175</Url>
-      <Description>TMFEV-885672295-4175</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100370F783D856BE247B308870A0815A245" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="e59e6bd7546e62b090aef4fb5ed9afb6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="15b42a90-06dd-4669-ae82-892e5974bb2f" xmlns:ns3="93d2b372-37bc-474e-a2f6-e237b07f4f3a" xmlns:ns4="2d89f73c-94c0-4155-aa8d-969ee56d6579" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4ca942eca7b8d364d6ad20a4d456e115" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="15b42a90-06dd-4669-ae82-892e5974bb2f"/>
@@ -1652,18 +1650,34 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="93d2b372-37bc-474e-a2f6-e237b07f4f3a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_dlc_DocId xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f">TMFEV-885672295-4175</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f">
+      <Url>https://tmfev.sharepoint.com/sites/tmf/mi-i/_layouts/15/DocIdRedir.aspx?ID=TMFEV-885672295-4175</Url>
+      <Description>TMFEV-885672295-4175</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1817AC26-B6E2-4C47-BB33-95CC1107F6F8}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08B8B0EA-3BDF-4954-AE09-AB5AAF359A99}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1817AC26-B6E2-4C47-BB33-95CC1107F6F8}"/>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24E64479-D726-4AB8-A716-1F18B611E8E6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAB6B2F1-2C78-4FE6-AF5B-CDBBCB8A75BF}"/>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAB6B2F1-2C78-4FE6-AF5B-CDBBCB8A75BF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24E64479-D726-4AB8-A716-1F18B611E8E6}"/>
 </file>
</xml_diff>

<commit_message>
Refine fallvignette export values refs #1328
</commit_message>
<xml_diff>
--- a/R-dataprocessor/submodules/manual_start/Fallvignette_Process_Evaluation/R-Fallvignette_Process_Evaluation/inst/extdata/WP8MRP_Liste_Daten_Mapping20260722.xlsx
+++ b/R-dataprocessor/submodules/manual_start/Fallvignette_Process_Evaluation/R-Fallvignette_Process_Evaluation/inst/extdata/WP8MRP_Liste_Daten_Mapping20260722.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{EE6A06D7-04C5-4693-89AC-F1482AA91ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E97DF81-D74D-4470-8A66-A9D79154D81D}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{EE6A06D7-04C5-4693-89AC-F1482AA91ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E313BC3E-37A0-4B6A-8EF9-7F135C944E00}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="57">
   <si>
     <t>Fallvignette</t>
   </si>
@@ -196,114 +196,6 @@
     <t>ret_gewiss_grund_abl_klin1_neg</t>
   </si>
   <si>
-    <t>wp8_ret_massn_am___1</t>
-  </si>
-  <si>
-    <t>ret_massn_am1___1</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_am___2</t>
-  </si>
-  <si>
-    <t>ret_massn_am1___2</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_am___3</t>
-  </si>
-  <si>
-    <t>ret_massn_am1___3</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_am___4</t>
-  </si>
-  <si>
-    <t>ret_massn_am1___4</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_am___5</t>
-  </si>
-  <si>
-    <t>ret_massn_am1___5</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_am___6</t>
-  </si>
-  <si>
-    <t>ret_massn_am1___6</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_am___7</t>
-  </si>
-  <si>
-    <t>ret_massn_am1___7</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_am___8</t>
-  </si>
-  <si>
-    <t>ret_massn_am1___8</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_am___9</t>
-  </si>
-  <si>
-    <t>ret_massn_am1___9</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_am___10</t>
-  </si>
-  <si>
-    <t>ret_massn_am1___10</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_orga___1</t>
-  </si>
-  <si>
-    <t>ret_massn_orga1___1</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_orga___2</t>
-  </si>
-  <si>
-    <t>ret_massn_orga1___2</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_orga___3</t>
-  </si>
-  <si>
-    <t>ret_massn_orga1___3</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_orga___4</t>
-  </si>
-  <si>
-    <t>ret_massn_orga1___4</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_orga___5</t>
-  </si>
-  <si>
-    <t>ret_massn_orga1___5</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_orga___6</t>
-  </si>
-  <si>
-    <t>ret_massn_orga1___6</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_orga___7</t>
-  </si>
-  <si>
-    <t>ret_massn_orga1___7</t>
-  </si>
-  <si>
-    <t>wp8_ret_massn_orga___8</t>
-  </si>
-  <si>
-    <t>ret_massn_orga1___8</t>
-  </si>
-  <si>
     <t>wp8_ret_notiz</t>
   </si>
   <si>
@@ -311,79 +203,25 @@
   </si>
   <si>
     <t>ret_gewissheit2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ret_gewiss_grund2_abl_01 </t>
+  </si>
+  <si>
+    <t>ret_gewiss_grund_abl_klin2</t>
+  </si>
+  <si>
+    <t>ret_gewiss_grund_abl_klin2_neg</t>
+  </si>
+  <si>
+    <t>ret_notiz2</t>
+  </si>
+  <si>
+    <t>mrp_auswahl_complete</t>
   </si>
   <si>
     <t>Ein retMRP kann zwei Bewertungen haben,
 Die je eine eigene Zeile bekommen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ret_gewiss_grund2_abl_01 </t>
-  </si>
-  <si>
-    <t>ret_gewiss_grund_abl_klin2</t>
-  </si>
-  <si>
-    <t>ret_gewiss_grund_abl_klin2_neg</t>
-  </si>
-  <si>
-    <t>ret_massn_am2___1</t>
-  </si>
-  <si>
-    <t>ret_massn_am2___2</t>
-  </si>
-  <si>
-    <t>ret_massn_am2___3</t>
-  </si>
-  <si>
-    <t>ret_massn_am2___4</t>
-  </si>
-  <si>
-    <t>ret_massn_am2___5</t>
-  </si>
-  <si>
-    <t>ret_massn_am2___6</t>
-  </si>
-  <si>
-    <t>ret_massn_am2___7</t>
-  </si>
-  <si>
-    <t>ret_massn_am2___8</t>
-  </si>
-  <si>
-    <t>ret_massn_am2___9</t>
-  </si>
-  <si>
-    <t>ret_massn_am2___10</t>
-  </si>
-  <si>
-    <t>ret_massn_orga2___1</t>
-  </si>
-  <si>
-    <t>ret_massn_orga2___2</t>
-  </si>
-  <si>
-    <t>ret_massn_orga2___3</t>
-  </si>
-  <si>
-    <t>ret_massn_orga2___4</t>
-  </si>
-  <si>
-    <t>ret_massn_orga2___5</t>
-  </si>
-  <si>
-    <t>ret_massn_orga2___6</t>
-  </si>
-  <si>
-    <t>ret_massn_orga2___7</t>
-  </si>
-  <si>
-    <t>ret_massn_orga2___8</t>
-  </si>
-  <si>
-    <t>ret_notiz2</t>
-  </si>
-  <si>
-    <t>mrp_auswahl_complete</t>
   </si>
   <si>
     <t>Select wenn Broad Consent und (ret_gewiss_grund1_abl_01 und/oder ret_gewiss_grund2_abl_01 =3)</t>
@@ -908,7 +746,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -916,7 +754,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -924,7 +762,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>38</v>
       </c>
@@ -932,7 +770,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>40</v>
       </c>
@@ -940,7 +778,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>42</v>
       </c>
@@ -948,7 +786,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:3">
       <c r="A22" t="s">
         <v>44</v>
       </c>
@@ -956,7 +794,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>46</v>
       </c>
@@ -964,353 +802,71 @@
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:3">
       <c r="A24" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" t="s">
         <v>48</v>
       </c>
-      <c r="B24" t="s">
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
-      <c r="A25" t="s">
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" t="s">
         <v>50</v>
       </c>
-      <c r="B25" t="s">
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
+        <v>44</v>
+      </c>
+      <c r="B27" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
-      <c r="A26" t="s">
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" t="s">
         <v>52</v>
       </c>
-      <c r="B26" t="s">
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="27" spans="1:2">
-      <c r="A27" t="s">
+      <c r="C29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="4:4" ht="24">
+      <c r="D42" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B27" t="s">
+    </row>
+    <row r="43" spans="4:4" ht="12.75"/>
+    <row r="71" spans="2:4">
+      <c r="B71" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="28" spans="1:2">
-      <c r="A28" t="s">
+      <c r="D71" t="s">
         <v>56</v>
-      </c>
-      <c r="B28" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2">
-      <c r="A29" t="s">
-        <v>58</v>
-      </c>
-      <c r="B29" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2">
-      <c r="A30" t="s">
-        <v>60</v>
-      </c>
-      <c r="B30" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2">
-      <c r="A31" t="s">
-        <v>62</v>
-      </c>
-      <c r="B31" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2">
-      <c r="A32" t="s">
-        <v>64</v>
-      </c>
-      <c r="B32" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4">
-      <c r="A33" t="s">
-        <v>66</v>
-      </c>
-      <c r="B33" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" t="s">
-        <v>68</v>
-      </c>
-      <c r="B34" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" t="s">
-        <v>70</v>
-      </c>
-      <c r="B35" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4">
-      <c r="A36" t="s">
-        <v>72</v>
-      </c>
-      <c r="B36" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4">
-      <c r="A37" t="s">
-        <v>74</v>
-      </c>
-      <c r="B37" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" t="s">
-        <v>76</v>
-      </c>
-      <c r="B38" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" t="s">
-        <v>78</v>
-      </c>
-      <c r="B39" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" t="s">
-        <v>80</v>
-      </c>
-      <c r="B40" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4">
-      <c r="A41" t="s">
-        <v>82</v>
-      </c>
-      <c r="B41" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="24">
-      <c r="A42" t="s">
-        <v>38</v>
-      </c>
-      <c r="B42" t="s">
-        <v>84</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="12.75">
-      <c r="A43" t="s">
-        <v>40</v>
-      </c>
-      <c r="B43" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4">
-      <c r="A44" t="s">
-        <v>42</v>
-      </c>
-      <c r="B44" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4">
-      <c r="A45" t="s">
-        <v>44</v>
-      </c>
-      <c r="B45" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4">
-      <c r="A46" t="s">
-        <v>46</v>
-      </c>
-      <c r="B46" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4">
-      <c r="A47" t="s">
-        <v>48</v>
-      </c>
-      <c r="B47" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4">
-      <c r="A48" t="s">
-        <v>50</v>
-      </c>
-      <c r="B48" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2">
-      <c r="A49" t="s">
-        <v>52</v>
-      </c>
-      <c r="B49" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2">
-      <c r="A50" t="s">
-        <v>54</v>
-      </c>
-      <c r="B50" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2">
-      <c r="A51" t="s">
-        <v>56</v>
-      </c>
-      <c r="B51" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2">
-      <c r="A52" t="s">
-        <v>58</v>
-      </c>
-      <c r="B52" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2">
-      <c r="A53" t="s">
-        <v>60</v>
-      </c>
-      <c r="B53" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2">
-      <c r="A54" t="s">
-        <v>62</v>
-      </c>
-      <c r="B54" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2">
-      <c r="A55" t="s">
-        <v>64</v>
-      </c>
-      <c r="B55" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2">
-      <c r="A56" t="s">
-        <v>66</v>
-      </c>
-      <c r="B56" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2">
-      <c r="A57" t="s">
-        <v>68</v>
-      </c>
-      <c r="B57" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2">
-      <c r="A58" t="s">
-        <v>70</v>
-      </c>
-      <c r="B58" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2">
-      <c r="A59" t="s">
-        <v>72</v>
-      </c>
-      <c r="B59" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2">
-      <c r="A60" t="s">
-        <v>74</v>
-      </c>
-      <c r="B60" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2">
-      <c r="A61" t="s">
-        <v>76</v>
-      </c>
-      <c r="B61" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2">
-      <c r="A62" t="s">
-        <v>78</v>
-      </c>
-      <c r="B62" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2">
-      <c r="A63" t="s">
-        <v>80</v>
-      </c>
-      <c r="B63" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2">
-      <c r="A64" t="s">
-        <v>82</v>
-      </c>
-      <c r="B64" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4">
-      <c r="A65" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4">
-      <c r="B71" t="s">
-        <v>109</v>
-      </c>
-      <c r="D71" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="98" spans="3:3">
       <c r="C98" t="s">
-        <v>108</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1336,53 +892,19 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="93d2b372-37bc-474e-a2f6-e237b07f4f3a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_dlc_DocId xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f">TMFEV-885672295-4175</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f">
+      <Url>https://tmfev.sharepoint.com/sites/tmf/mi-i/_layouts/15/DocIdRedir.aspx?ID=TMFEV-885672295-4175</Url>
+      <Description>TMFEV-885672295-4175</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1651,19 +1173,53 @@
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="93d2b372-37bc-474e-a2f6-e237b07f4f3a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_dlc_DocId xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f">TMFEV-885672295-4175</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f">
-      <Url>https://tmfev.sharepoint.com/sites/tmf/mi-i/_layouts/15/DocIdRedir.aspx?ID=TMFEV-885672295-4175</Url>
-      <Description>TMFEV-885672295-4175</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1671,7 +1227,7 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08B8B0EA-3BDF-4954-AE09-AB5AAF359A99}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24E64479-D726-4AB8-A716-1F18B611E8E6}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1679,5 +1235,5 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24E64479-D726-4AB8-A716-1F18B611E8E6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08B8B0EA-3BDF-4954-AE09-AB5AAF359A99}"/>
 </file>
</xml_diff>

<commit_message>
Normalize fallvignette REDCap fields refs #1328
</commit_message>
<xml_diff>
--- a/R-dataprocessor/submodules/manual_start/Fallvignette_Process_Evaluation/R-Fallvignette_Process_Evaluation/inst/extdata/WP8MRP_Liste_Daten_Mapping20260722.xlsx
+++ b/R-dataprocessor/submodules/manual_start/Fallvignette_Process_Evaluation/R-Fallvignette_Process_Evaluation/inst/extdata/WP8MRP_Liste_Daten_Mapping20260722.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30413"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{EE6A06D7-04C5-4693-89AC-F1482AA91ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E313BC3E-37A0-4B6A-8EF9-7F135C944E00}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{EE6A06D7-04C5-4693-89AC-F1482AA91ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE2BCB6E-6C63-4317-A6AC-B181C8ECA664}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -187,13 +187,13 @@
     <t>wp8_ret_gewiss_grund_abl_klin</t>
   </si>
   <si>
-    <t xml:space="preserve">ret_gewiss_grund_abl_klin1 </t>
-  </si>
-  <si>
-    <t>wp8_ret_gewiss_grund_abl_klin_neg</t>
-  </si>
-  <si>
-    <t>ret_gewiss_grund_abl_klin1_neg</t>
+    <t>ret_gewiss_grund_abl_klin1</t>
+  </si>
+  <si>
+    <t>wp8_ret_gewiss_grund_abl_klin_neg___1</t>
+  </si>
+  <si>
+    <t>ret_gewiss_grund_abl_klin1_neg___1</t>
   </si>
   <si>
     <t>wp8_ret_notiz</t>
@@ -211,7 +211,7 @@
     <t>ret_gewiss_grund_abl_klin2</t>
   </si>
   <si>
-    <t>ret_gewiss_grund_abl_klin2_neg</t>
+    <t>ret_gewiss_grund_abl_klin2_neg___1</t>
   </si>
   <si>
     <t>ret_notiz2</t>
@@ -883,15 +883,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f" xsi:nil="true"/>
@@ -907,7 +898,66 @@
 </p:properties>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100370F783D856BE247B308870A0815A245" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="e59e6bd7546e62b090aef4fb5ed9afb6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="15b42a90-06dd-4669-ae82-892e5974bb2f" xmlns:ns3="93d2b372-37bc-474e-a2f6-e237b07f4f3a" xmlns:ns4="2d89f73c-94c0-4155-aa8d-969ee56d6579" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4ca942eca7b8d364d6ad20a4d456e115" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="15b42a90-06dd-4669-ae82-892e5974bb2f"/>
@@ -1172,68 +1222,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24E64479-D726-4AB8-A716-1F18B611E8E6}"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1817AC26-B6E2-4C47-BB33-95CC1107F6F8}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24E64479-D726-4AB8-A716-1F18B611E8E6}"/>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAB6B2F1-2C78-4FE6-AF5B-CDBBCB8A75BF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08B8B0EA-3BDF-4954-AE09-AB5AAF359A99}"/>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08B8B0EA-3BDF-4954-AE09-AB5AAF359A99}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAB6B2F1-2C78-4FE6-AF5B-CDBBCB8A75BF}"/>
 </file>
</xml_diff>